<commit_message>
Added a Criticality/Redundancy/Reliability Profile. Made shop center of gravity calculation along with displacement. Also edited Plugin guide
</commit_message>
<xml_diff>
--- a/Properties.xlsx
+++ b/Properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kkoch28\Downloads\NAVSEA RESEARCH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B34EEF88-0459-424E-BEB9-13830E1F1976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D74DB7C-B253-4D50-B661-F366B94FC365}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="8595" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -735,20 +735,19 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <f t="shared" ref="B5:E39" ca="1" si="0">RANDBETWEEN(1,100)</f>
-        <v>52</v>
+        <f ca="1">RANDBETWEEN(20,750)</f>
+        <v>378</v>
       </c>
       <c r="C5">
-        <f t="shared" ref="C5:F5" ca="1" si="1">RANDBETWEEN(1,100)</f>
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="D5">
-        <f t="shared" ca="1" si="1"/>
-        <v>21</v>
+        <f t="shared" ref="D5:D13" ca="1" si="0">RANDBETWEEN(1,5)</f>
+        <v>5</v>
       </c>
       <c r="E5">
-        <f t="shared" ca="1" si="1"/>
-        <v>26</v>
+        <f t="shared" ref="E5:E39" ca="1" si="1">RANDBETWEEN(-10,10)</f>
+        <v>-1</v>
       </c>
       <c r="F5" t="s">
         <v>57</v>
@@ -771,20 +770,20 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <f t="shared" ref="B6:B39" ca="1" si="2">RANDBETWEEN(20,750)</f>
+        <v>452</v>
       </c>
       <c r="C6">
-        <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <f t="shared" ref="B5:E39" ca="1" si="3">RANDBETWEEN(1,100)</f>
+        <v>68</v>
       </c>
       <c r="D6">
         <f t="shared" ca="1" si="0"/>
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <f t="shared" ca="1" si="0"/>
-        <v>38</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>1</v>
       </c>
       <c r="F6" t="s">
         <v>57</v>
@@ -807,20 +806,20 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>730</v>
       </c>
       <c r="C7">
-        <f t="shared" ca="1" si="0"/>
-        <v>7</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>24</v>
       </c>
       <c r="D7">
         <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="E7">
-        <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>7</v>
       </c>
       <c r="F7" t="s">
         <v>57</v>
@@ -843,20 +842,20 @@
         <v>0</v>
       </c>
       <c r="B8">
-        <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>700</v>
       </c>
       <c r="C8">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" ca="1" si="3"/>
         <v>37</v>
       </c>
       <c r="D8">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>5</v>
       </c>
       <c r="E8">
-        <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-8</v>
       </c>
       <c r="F8" t="s">
         <v>57</v>
@@ -865,8 +864,8 @@
         <v>57</v>
       </c>
       <c r="H8">
-        <f t="shared" ref="H6:H10" ca="1" si="2">RANDBETWEEN(1,15)</f>
-        <v>2</v>
+        <f t="shared" ref="H8:H10" ca="1" si="4">RANDBETWEEN(1,15)</f>
+        <v>13</v>
       </c>
       <c r="I8">
         <v>0.7</v>
@@ -881,20 +880,20 @@
         <v>1</v>
       </c>
       <c r="B9">
-        <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>294</v>
       </c>
       <c r="C9">
-        <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>76</v>
       </c>
       <c r="D9">
-        <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <f ca="1">RANDBETWEEN(1,5)</f>
+        <v>5</v>
       </c>
       <c r="E9">
-        <f t="shared" ca="1" si="0"/>
-        <v>5</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>10</v>
       </c>
       <c r="F9" t="s">
         <v>57</v>
@@ -903,14 +902,14 @@
         <v>57</v>
       </c>
       <c r="H9">
-        <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>10</v>
       </c>
       <c r="I9">
         <v>0.2</v>
       </c>
       <c r="J9" t="b">
-        <f t="shared" ref="J9:J10" ca="1" si="3">IF(RAND()&lt;0.5,TRUE,FALSE)</f>
+        <f t="shared" ref="J9:J10" ca="1" si="5">IF(RAND()&lt;0.5,TRUE,FALSE)</f>
         <v>0</v>
       </c>
     </row>
@@ -919,20 +918,20 @@
         <v>2</v>
       </c>
       <c r="B10">
-        <f t="shared" ca="1" si="0"/>
-        <v>54</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>344</v>
       </c>
       <c r="C10">
-        <f t="shared" ca="1" si="0"/>
-        <v>64</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>57</v>
       </c>
       <c r="D10">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="E10">
-        <f t="shared" ca="1" si="0"/>
-        <v>37</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-5</v>
       </c>
       <c r="F10" t="s">
         <v>57</v>
@@ -941,15 +940,15 @@
         <v>57</v>
       </c>
       <c r="H10">
-        <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>11</v>
       </c>
       <c r="I10">
         <v>0.9</v>
       </c>
       <c r="J10" t="b">
-        <f t="shared" ca="1" si="3"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -957,20 +956,20 @@
         <v>3</v>
       </c>
       <c r="B11">
-        <f t="shared" ca="1" si="0"/>
-        <v>54</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>488</v>
       </c>
       <c r="C11">
-        <f t="shared" ca="1" si="0"/>
-        <v>69</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>15</v>
       </c>
       <c r="D11">
         <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="E11">
-        <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
       </c>
       <c r="F11">
         <v>7</v>
@@ -993,20 +992,20 @@
         <v>59</v>
       </c>
       <c r="B12">
-        <f t="shared" ca="1" si="0"/>
-        <v>88</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>430</v>
       </c>
       <c r="C12">
-        <f t="shared" ca="1" si="0"/>
-        <v>17</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>14</v>
       </c>
       <c r="D12">
         <f t="shared" ca="1" si="0"/>
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="E12">
-        <f t="shared" ca="1" si="0"/>
-        <v>65</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>5</v>
       </c>
       <c r="F12">
         <v>20</v>
@@ -1029,20 +1028,20 @@
         <v>58</v>
       </c>
       <c r="B13">
+        <f t="shared" ca="1" si="2"/>
+        <v>674</v>
+      </c>
+      <c r="C13">
+        <f t="shared" ca="1" si="3"/>
+        <v>58</v>
+      </c>
+      <c r="D13">
         <f t="shared" ca="1" si="0"/>
         <v>3</v>
       </c>
-      <c r="C13">
-        <f t="shared" ca="1" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="D13">
-        <f t="shared" ca="1" si="0"/>
-        <v>1</v>
-      </c>
       <c r="E13">
-        <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-2</v>
       </c>
       <c r="F13" t="s">
         <v>57</v>
@@ -1052,14 +1051,14 @@
       </c>
       <c r="H13">
         <f ca="1">RANDBETWEEN(1,15)</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I13">
         <v>0.15</v>
       </c>
       <c r="J13" t="b">
         <f ca="1">IF(RAND()&lt;0.5,TRUE,FALSE)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1067,20 +1066,20 @@
         <v>8</v>
       </c>
       <c r="B14">
-        <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>619</v>
       </c>
       <c r="C14">
-        <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>48</v>
       </c>
       <c r="D14">
-        <f t="shared" ca="1" si="0"/>
-        <v>57</v>
+        <f ca="1">RANDBETWEEN(1,30)</f>
+        <v>20</v>
       </c>
       <c r="E14">
-        <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-6</v>
       </c>
       <c r="F14">
         <v>15</v>
@@ -1090,14 +1089,14 @@
       </c>
       <c r="H14">
         <f ca="1">RANDBETWEEN(1,15)</f>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I14">
         <v>0.15</v>
       </c>
       <c r="J14" t="b">
         <f ca="1">IF(RAND()&lt;0.5,TRUE,FALSE)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1105,20 +1104,20 @@
         <v>9</v>
       </c>
       <c r="B15">
-        <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>683</v>
       </c>
       <c r="C15">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" ca="1" si="3"/>
+        <v>24</v>
+      </c>
+      <c r="D15">
+        <f t="shared" ref="D15:D39" ca="1" si="6">RANDBETWEEN(1,30)</f>
         <v>17</v>
       </c>
-      <c r="D15">
-        <f t="shared" ca="1" si="0"/>
-        <v>54</v>
-      </c>
       <c r="E15">
-        <f t="shared" ca="1" si="0"/>
-        <v>25</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>6</v>
       </c>
       <c r="F15">
         <v>12</v>
@@ -1141,20 +1140,20 @@
         <v>10</v>
       </c>
       <c r="B16">
-        <f t="shared" ca="1" si="0"/>
-        <v>64</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>291</v>
       </c>
       <c r="C16">
-        <f t="shared" ca="1" si="0"/>
-        <v>21</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>44</v>
       </c>
       <c r="D16">
-        <f t="shared" ca="1" si="0"/>
-        <v>76</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>26</v>
       </c>
       <c r="E16">
-        <f t="shared" ca="1" si="0"/>
-        <v>50</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>8</v>
       </c>
       <c r="F16" t="s">
         <v>57</v>
@@ -1164,14 +1163,14 @@
       </c>
       <c r="H16">
         <f ca="1">RANDBETWEEN(1,15)</f>
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I16">
         <v>0.3</v>
       </c>
       <c r="J16" t="b">
         <f ca="1">IF(RAND()&lt;0.5,TRUE,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1179,20 +1178,20 @@
         <v>11</v>
       </c>
       <c r="B17">
-        <f t="shared" ca="1" si="0"/>
-        <v>8</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>398</v>
       </c>
       <c r="C17">
-        <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>77</v>
       </c>
       <c r="D17">
-        <f t="shared" ca="1" si="0"/>
-        <v>57</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>6</v>
       </c>
       <c r="E17">
-        <f t="shared" ca="1" si="0"/>
-        <v>35</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>9</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>57</v>
@@ -1201,15 +1200,15 @@
         <v>57</v>
       </c>
       <c r="H17">
-        <f t="shared" ref="H17:H39" ca="1" si="4">RANDBETWEEN(1,15)</f>
-        <v>11</v>
+        <f t="shared" ref="H17:H39" ca="1" si="7">RANDBETWEEN(1,15)</f>
+        <v>15</v>
       </c>
       <c r="I17">
         <v>0.15</v>
       </c>
       <c r="J17" t="b">
-        <f t="shared" ref="J17:J39" ca="1" si="5">IF(RAND()&lt;0.5,TRUE,FALSE)</f>
-        <v>1</v>
+        <f t="shared" ref="J17:J39" ca="1" si="8">IF(RAND()&lt;0.5,TRUE,FALSE)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1217,20 +1216,20 @@
         <v>12</v>
       </c>
       <c r="B18">
-        <f t="shared" ca="1" si="0"/>
-        <v>58</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>551</v>
       </c>
       <c r="C18">
-        <f t="shared" ca="1" si="0"/>
-        <v>59</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>22</v>
       </c>
       <c r="D18">
-        <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>27</v>
       </c>
       <c r="E18">
-        <f t="shared" ca="1" si="0"/>
-        <v>19</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>57</v>
@@ -1239,15 +1238,15 @@
         <v>57</v>
       </c>
       <c r="H18">
-        <f t="shared" ca="1" si="4"/>
-        <v>13</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>5</v>
       </c>
       <c r="I18">
         <v>0.25</v>
       </c>
       <c r="J18" t="b">
-        <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1255,20 +1254,20 @@
         <v>13</v>
       </c>
       <c r="B19">
-        <f t="shared" ca="1" si="0"/>
-        <v>39</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>284</v>
       </c>
       <c r="C19">
-        <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>95</v>
       </c>
       <c r="D19">
-        <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>25</v>
       </c>
       <c r="E19">
-        <f t="shared" ca="1" si="0"/>
-        <v>75</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-3</v>
       </c>
       <c r="F19" t="s">
         <v>57</v>
@@ -1278,13 +1277,13 @@
       </c>
       <c r="H19">
         <f ca="1">RANDBETWEEN(1,15)</f>
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="I19">
         <v>0.35</v>
       </c>
       <c r="J19" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -1293,20 +1292,20 @@
         <v>14</v>
       </c>
       <c r="B20">
-        <f t="shared" ca="1" si="0"/>
-        <v>42</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>76</v>
       </c>
       <c r="C20">
-        <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>79</v>
       </c>
       <c r="D20">
-        <f t="shared" ca="1" si="0"/>
-        <v>30</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>8</v>
       </c>
       <c r="E20">
-        <f t="shared" ca="1" si="0"/>
-        <v>58</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-8</v>
       </c>
       <c r="F20" t="s">
         <v>57</v>
@@ -1315,15 +1314,15 @@
         <v>57</v>
       </c>
       <c r="H20">
-        <f t="shared" ca="1" si="4"/>
-        <v>13</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>3</v>
       </c>
       <c r="I20">
         <v>0.85</v>
       </c>
       <c r="J20" t="b">
-        <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1331,20 +1330,20 @@
         <v>15</v>
       </c>
       <c r="B21">
-        <f t="shared" ca="1" si="0"/>
-        <v>56</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>642</v>
       </c>
       <c r="C21">
-        <f t="shared" ca="1" si="0"/>
-        <v>25</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>85</v>
       </c>
       <c r="D21">
-        <f t="shared" ca="1" si="0"/>
-        <v>97</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>24</v>
       </c>
       <c r="E21">
-        <f t="shared" ca="1" si="0"/>
-        <v>9</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-3</v>
       </c>
       <c r="F21" t="s">
         <v>57</v>
@@ -1353,15 +1352,15 @@
         <v>57</v>
       </c>
       <c r="H21">
-        <f t="shared" ca="1" si="4"/>
-        <v>10</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>5</v>
       </c>
       <c r="I21">
         <v>0.75</v>
       </c>
       <c r="J21" t="b">
-        <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1369,20 +1368,20 @@
         <v>16</v>
       </c>
       <c r="B22">
-        <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>437</v>
       </c>
       <c r="C22">
-        <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>19</v>
       </c>
       <c r="D22">
-        <f t="shared" ca="1" si="0"/>
-        <v>48</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>18</v>
       </c>
       <c r="E22">
-        <f t="shared" ca="1" si="0"/>
-        <v>46</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
       </c>
       <c r="F22" t="s">
         <v>57</v>
@@ -1391,14 +1390,14 @@
         <v>57</v>
       </c>
       <c r="H22">
-        <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>11</v>
       </c>
       <c r="I22">
         <v>0.3</v>
       </c>
       <c r="J22" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1407,20 +1406,20 @@
         <v>17</v>
       </c>
       <c r="B23">
-        <f t="shared" ca="1" si="0"/>
-        <v>27</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>223</v>
       </c>
       <c r="C23">
-        <f t="shared" ca="1" si="0"/>
-        <v>34</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>70</v>
       </c>
       <c r="D23">
-        <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>12</v>
       </c>
       <c r="E23">
-        <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
       </c>
       <c r="F23" t="s">
         <v>57</v>
@@ -1429,14 +1428,14 @@
         <v>57</v>
       </c>
       <c r="H23">
-        <f t="shared" ca="1" si="4"/>
-        <v>9</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>6</v>
       </c>
       <c r="I23">
         <v>0.15</v>
       </c>
       <c r="J23" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1445,20 +1444,20 @@
         <v>18</v>
       </c>
       <c r="B24">
-        <f t="shared" ca="1" si="0"/>
-        <v>49</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>264</v>
       </c>
       <c r="C24">
-        <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>9</v>
       </c>
       <c r="D24">
-        <f t="shared" ca="1" si="0"/>
-        <v>86</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>28</v>
       </c>
       <c r="E24">
-        <f t="shared" ca="1" si="0"/>
-        <v>71</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-4</v>
       </c>
       <c r="F24" t="s">
         <v>57</v>
@@ -1467,14 +1466,14 @@
         <v>57</v>
       </c>
       <c r="H24">
-        <f t="shared" ca="1" si="4"/>
-        <v>14</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>7</v>
       </c>
       <c r="I24">
         <v>0.25</v>
       </c>
       <c r="J24" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1483,36 +1482,36 @@
         <v>19</v>
       </c>
       <c r="B25">
-        <f t="shared" ca="1" si="0"/>
-        <v>10</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>356</v>
       </c>
       <c r="C25">
-        <f t="shared" ca="1" si="0"/>
-        <v>71</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>30</v>
       </c>
       <c r="D25">
-        <f t="shared" ca="1" si="0"/>
-        <v>21</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>14</v>
       </c>
       <c r="E25">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" ca="1" si="1"/>
+        <v>-6</v>
+      </c>
+      <c r="F25" t="s">
+        <v>57</v>
+      </c>
+      <c r="G25" t="s">
+        <v>57</v>
+      </c>
+      <c r="H25">
+        <f t="shared" ca="1" si="7"/>
         <v>6</v>
-      </c>
-      <c r="F25" t="s">
-        <v>57</v>
-      </c>
-      <c r="G25" t="s">
-        <v>57</v>
-      </c>
-      <c r="H25">
-        <f t="shared" ca="1" si="4"/>
-        <v>15</v>
       </c>
       <c r="I25">
         <v>0.35</v>
       </c>
       <c r="J25" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -1521,20 +1520,20 @@
         <v>20</v>
       </c>
       <c r="B26">
-        <f t="shared" ca="1" si="0"/>
-        <v>71</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>90</v>
       </c>
       <c r="C26">
-        <f t="shared" ca="1" si="0"/>
-        <v>38</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>82</v>
       </c>
       <c r="D26">
-        <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>14</v>
       </c>
       <c r="E26">
-        <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>5</v>
       </c>
       <c r="F26" t="s">
         <v>57</v>
@@ -1543,14 +1542,14 @@
         <v>57</v>
       </c>
       <c r="H26">
-        <f t="shared" ca="1" si="4"/>
-        <v>15</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>13</v>
       </c>
       <c r="I26">
         <v>0.85</v>
       </c>
       <c r="J26" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -1559,20 +1558,20 @@
         <v>21</v>
       </c>
       <c r="B27">
-        <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>50</v>
       </c>
       <c r="C27">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" ca="1" si="3"/>
+        <v>84</v>
+      </c>
+      <c r="D27">
+        <f t="shared" ca="1" si="6"/>
         <v>29</v>
       </c>
-      <c r="D27">
-        <f t="shared" ca="1" si="0"/>
-        <v>44</v>
-      </c>
       <c r="E27">
-        <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-2</v>
       </c>
       <c r="F27" t="s">
         <v>57</v>
@@ -1581,15 +1580,15 @@
         <v>57</v>
       </c>
       <c r="H27">
-        <f t="shared" ca="1" si="4"/>
-        <v>14</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>1</v>
       </c>
       <c r="I27">
         <v>0.75</v>
       </c>
       <c r="J27" t="b">
-        <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1597,20 +1596,20 @@
         <v>22</v>
       </c>
       <c r="B28">
-        <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>25</v>
       </c>
       <c r="C28">
-        <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>59</v>
       </c>
       <c r="D28">
-        <f t="shared" ca="1" si="0"/>
-        <v>43</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>8</v>
       </c>
       <c r="E28">
-        <f t="shared" ca="1" si="0"/>
-        <v>7</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-6</v>
       </c>
       <c r="F28" t="s">
         <v>57</v>
@@ -1619,14 +1618,14 @@
         <v>57</v>
       </c>
       <c r="H28">
-        <f t="shared" ca="1" si="4"/>
-        <v>5</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>9</v>
       </c>
       <c r="I28">
         <v>0.3</v>
       </c>
       <c r="J28" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1635,20 +1634,20 @@
         <v>23</v>
       </c>
       <c r="B29">
-        <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>340</v>
       </c>
       <c r="C29">
-        <f t="shared" ca="1" si="0"/>
-        <v>79</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>10</v>
       </c>
       <c r="D29">
-        <f t="shared" ca="1" si="0"/>
-        <v>78</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>19</v>
       </c>
       <c r="E29">
-        <f t="shared" ca="1" si="0"/>
-        <v>64</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-1</v>
       </c>
       <c r="F29" t="s">
         <v>57</v>
@@ -1657,14 +1656,14 @@
         <v>57</v>
       </c>
       <c r="H29">
-        <f t="shared" ca="1" si="4"/>
-        <v>12</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>2</v>
       </c>
       <c r="I29">
         <v>0.15</v>
       </c>
       <c r="J29" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1673,20 +1672,20 @@
         <v>24</v>
       </c>
       <c r="B30">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" ca="1" si="2"/>
+        <v>25</v>
+      </c>
+      <c r="C30">
+        <f t="shared" ca="1" si="3"/>
         <v>81</v>
       </c>
-      <c r="C30">
-        <f t="shared" ca="1" si="0"/>
-        <v>39</v>
-      </c>
       <c r="D30">
-        <f t="shared" ca="1" si="0"/>
-        <v>49</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>10</v>
       </c>
       <c r="E30">
-        <f t="shared" ca="1" si="0"/>
-        <v>71</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>10</v>
       </c>
       <c r="F30" t="s">
         <v>57</v>
@@ -1695,15 +1694,15 @@
         <v>57</v>
       </c>
       <c r="H30">
-        <f t="shared" ca="1" si="4"/>
-        <v>10</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>3</v>
       </c>
       <c r="I30">
         <v>0.25</v>
       </c>
       <c r="J30" t="b">
-        <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1711,20 +1710,20 @@
         <v>25</v>
       </c>
       <c r="B31">
-        <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>151</v>
       </c>
       <c r="C31">
-        <f t="shared" ca="1" si="0"/>
-        <v>49</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>21</v>
       </c>
       <c r="D31">
-        <f t="shared" ca="1" si="0"/>
-        <v>41</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>25</v>
       </c>
       <c r="E31">
-        <f t="shared" ca="1" si="0"/>
-        <v>9</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-3</v>
       </c>
       <c r="F31" t="s">
         <v>57</v>
@@ -1733,15 +1732,15 @@
         <v>57</v>
       </c>
       <c r="H31">
-        <f t="shared" ca="1" si="4"/>
-        <v>10</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>8</v>
       </c>
       <c r="I31">
         <v>0.35</v>
       </c>
       <c r="J31" t="b">
-        <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1749,20 +1748,20 @@
         <v>26</v>
       </c>
       <c r="B32">
-        <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>696</v>
       </c>
       <c r="C32">
-        <f t="shared" ca="1" si="0"/>
-        <v>17</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>7</v>
       </c>
       <c r="D32">
-        <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>22</v>
       </c>
       <c r="E32">
-        <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>9</v>
       </c>
       <c r="F32" t="s">
         <v>57</v>
@@ -1771,15 +1770,15 @@
         <v>57</v>
       </c>
       <c r="H32">
-        <f t="shared" ca="1" si="4"/>
-        <v>6</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>10</v>
       </c>
       <c r="I32">
         <v>0.85</v>
       </c>
       <c r="J32" t="b">
-        <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1787,20 +1786,20 @@
         <v>27</v>
       </c>
       <c r="B33">
-        <f t="shared" ca="1" si="0"/>
-        <v>18</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>92</v>
       </c>
       <c r="C33">
-        <f t="shared" ca="1" si="0"/>
-        <v>21</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>96</v>
       </c>
       <c r="D33">
-        <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>1</v>
       </c>
       <c r="E33">
-        <f t="shared" ca="1" si="0"/>
-        <v>5</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>8</v>
       </c>
       <c r="F33" t="s">
         <v>57</v>
@@ -1809,15 +1808,15 @@
         <v>57</v>
       </c>
       <c r="H33">
-        <f t="shared" ca="1" si="4"/>
-        <v>4</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>12</v>
       </c>
       <c r="I33">
         <v>0.75</v>
       </c>
       <c r="J33" t="b">
-        <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1825,20 +1824,20 @@
         <v>28</v>
       </c>
       <c r="B34">
-        <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>347</v>
       </c>
       <c r="C34">
-        <f t="shared" ca="1" si="0"/>
-        <v>24</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>3</v>
       </c>
       <c r="D34">
-        <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>15</v>
       </c>
       <c r="E34">
-        <f t="shared" ca="1" si="0"/>
-        <v>37</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>8</v>
       </c>
       <c r="F34" t="s">
         <v>57</v>
@@ -1847,14 +1846,14 @@
         <v>57</v>
       </c>
       <c r="H34">
-        <f t="shared" ca="1" si="4"/>
-        <v>11</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>13</v>
       </c>
       <c r="I34">
         <v>0.3</v>
       </c>
       <c r="J34" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -1863,20 +1862,20 @@
         <v>29</v>
       </c>
       <c r="B35">
-        <f t="shared" ca="1" si="0"/>
-        <v>11</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>63</v>
       </c>
       <c r="C35">
-        <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>8</v>
       </c>
       <c r="D35">
-        <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>5</v>
       </c>
       <c r="E35">
-        <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>1</v>
       </c>
       <c r="F35" t="s">
         <v>57</v>
@@ -1885,15 +1884,15 @@
         <v>57</v>
       </c>
       <c r="H35">
-        <f t="shared" ca="1" si="4"/>
-        <v>6</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>15</v>
       </c>
       <c r="I35">
         <v>0.15</v>
       </c>
       <c r="J35" t="b">
-        <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1901,20 +1900,20 @@
         <v>30</v>
       </c>
       <c r="B36">
-        <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>654</v>
       </c>
       <c r="C36">
-        <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>68</v>
       </c>
       <c r="D36">
-        <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>21</v>
       </c>
       <c r="E36">
-        <f t="shared" ca="1" si="0"/>
-        <v>7</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>2</v>
       </c>
       <c r="F36" t="s">
         <v>57</v>
@@ -1923,14 +1922,14 @@
         <v>57</v>
       </c>
       <c r="H36">
-        <f t="shared" ca="1" si="4"/>
-        <v>6</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>12</v>
       </c>
       <c r="I36">
         <v>0.25</v>
       </c>
       <c r="J36" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>1</v>
       </c>
     </row>
@@ -1939,20 +1938,20 @@
         <v>31</v>
       </c>
       <c r="B37">
-        <f t="shared" ca="1" si="0"/>
-        <v>67</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>118</v>
       </c>
       <c r="C37">
-        <f t="shared" ca="1" si="0"/>
-        <v>43</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>26</v>
       </c>
       <c r="D37">
-        <f t="shared" ca="1" si="0"/>
-        <v>44</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>26</v>
       </c>
       <c r="E37">
-        <f t="shared" ca="1" si="0"/>
-        <v>4</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-5</v>
       </c>
       <c r="F37" t="s">
         <v>57</v>
@@ -1961,14 +1960,14 @@
         <v>57</v>
       </c>
       <c r="H37">
-        <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>12</v>
       </c>
       <c r="I37">
         <v>0.35</v>
       </c>
       <c r="J37" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1977,20 +1976,20 @@
         <v>32</v>
       </c>
       <c r="B38">
-        <f t="shared" ca="1" si="0"/>
-        <v>5</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>593</v>
       </c>
       <c r="C38">
-        <f t="shared" ca="1" si="0"/>
-        <v>69</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>26</v>
       </c>
       <c r="D38">
-        <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>19</v>
       </c>
       <c r="E38">
-        <f t="shared" ca="1" si="0"/>
-        <v>38</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>7</v>
       </c>
       <c r="F38" t="s">
         <v>57</v>
@@ -1999,15 +1998,15 @@
         <v>57</v>
       </c>
       <c r="H38">
-        <f t="shared" ca="1" si="4"/>
-        <v>10</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>3</v>
       </c>
       <c r="I38">
         <v>0.85</v>
       </c>
       <c r="J38" t="b">
-        <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="8"/>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -2015,20 +2014,20 @@
         <v>33</v>
       </c>
       <c r="B39">
-        <f t="shared" ca="1" si="0"/>
-        <v>2</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>470</v>
       </c>
       <c r="C39">
-        <f t="shared" ca="1" si="0"/>
-        <v>8</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>15</v>
       </c>
       <c r="D39">
-        <f t="shared" ca="1" si="0"/>
-        <v>21</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>6</v>
       </c>
       <c r="E39">
-        <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>-3</v>
       </c>
       <c r="F39" t="s">
         <v>57</v>
@@ -2037,14 +2036,14 @@
         <v>57</v>
       </c>
       <c r="H39">
-        <f t="shared" ca="1" si="4"/>
-        <v>9</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>4</v>
       </c>
       <c r="I39">
         <v>0.75</v>
       </c>
       <c r="J39" t="b">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="8"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>